<commit_message>
Add charts for increase_budget
</commit_message>
<xml_diff>
--- a/tables_increase_budget.xlsx
+++ b/tables_increase_budget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Me\UofL\Data Analytics &amp; System Optimization (DASO)\MetroSafe Drone-Project\MetroSafe-UofL_Drone_Optimization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55DDF45F-1425-4114-9305-658EC75D229D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DAEA114-02C9-4818-8989-0B430E9A03AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -395,6 +395,7 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
+      <c r="F1" s="2"/>
       <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
@@ -419,6 +420,7 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="F2" s="2"/>
       <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
@@ -451,6 +453,7 @@
       <c r="E3" s="2">
         <v>1</v>
       </c>
+      <c r="F3" s="2"/>
       <c r="G3" s="2">
         <v>1</v>
       </c>
@@ -483,6 +486,7 @@
       <c r="E4" s="2">
         <v>2</v>
       </c>
+      <c r="F4" s="2"/>
       <c r="G4" s="2">
         <v>2</v>
       </c>
@@ -515,6 +519,7 @@
       <c r="E5" s="2">
         <v>3</v>
       </c>
+      <c r="F5" s="2"/>
       <c r="G5" s="2">
         <v>3</v>
       </c>
@@ -547,6 +552,7 @@
       <c r="E6" s="2">
         <v>4</v>
       </c>
+      <c r="F6" s="2"/>
       <c r="G6" s="2">
         <v>4</v>
       </c>
@@ -579,6 +585,7 @@
       <c r="E7" s="2">
         <v>5</v>
       </c>
+      <c r="F7" s="2"/>
       <c r="G7" s="2">
         <v>5</v>
       </c>
@@ -611,6 +618,7 @@
       <c r="E8" s="2">
         <v>6</v>
       </c>
+      <c r="F8" s="2"/>
       <c r="G8" s="2">
         <v>6</v>
       </c>
@@ -643,6 +651,7 @@
       <c r="E9" s="2">
         <v>7</v>
       </c>
+      <c r="F9" s="2"/>
       <c r="G9" s="2">
         <v>7</v>
       </c>
@@ -675,6 +684,7 @@
       <c r="E10" s="2">
         <v>7</v>
       </c>
+      <c r="F10" s="2"/>
       <c r="G10" s="2">
         <v>8</v>
       </c>
@@ -707,6 +717,7 @@
       <c r="E11" s="2">
         <v>7</v>
       </c>
+      <c r="F11" s="2"/>
       <c r="G11" s="2">
         <v>9</v>
       </c>
@@ -739,6 +750,7 @@
       <c r="E12" s="2">
         <v>7</v>
       </c>
+      <c r="F12" s="2"/>
       <c r="G12" s="2">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Include Compare Charts feature
</commit_message>
<xml_diff>
--- a/tables_increase_budget.xlsx
+++ b/tables_increase_budget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Me\UofL\Data Analytics &amp; System Optimization (DASO)\MetroSafe Drone-Project\MetroSafe-UofL_Drone_Optimization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DAEA114-02C9-4818-8989-0B430E9A03AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FBEC0BE-A064-4668-991D-17915B4B0B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -372,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>38.89</v>
+        <v>7.63</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
@@ -458,7 +458,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="2">
-        <v>16.670000000000002</v>
+        <v>7.63</v>
       </c>
       <c r="I3" s="2">
         <v>1</v>
@@ -475,23 +475,23 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>55.56</v>
+        <v>15.27</v>
       </c>
       <c r="C4" s="2">
         <v>2</v>
       </c>
       <c r="D4" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2">
         <v>2</v>
       </c>
       <c r="H4" s="2">
-        <v>27.78</v>
+        <v>15.27</v>
       </c>
       <c r="I4" s="2">
         <v>2</v>
@@ -508,23 +508,23 @@
         <v>3</v>
       </c>
       <c r="B5" s="2">
-        <v>66.67</v>
+        <v>22.9</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
       </c>
       <c r="D5" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2">
         <v>3</v>
       </c>
       <c r="H5" s="2">
-        <v>33.33</v>
+        <v>22.9</v>
       </c>
       <c r="I5" s="2">
         <v>3</v>
@@ -541,23 +541,23 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>77.78</v>
+        <v>30.53</v>
       </c>
       <c r="C6" s="2">
         <v>4</v>
       </c>
       <c r="D6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2">
         <v>4</v>
       </c>
       <c r="H6" s="2">
-        <v>38.89</v>
+        <v>29.01</v>
       </c>
       <c r="I6" s="2">
         <v>4</v>
@@ -574,32 +574,32 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>83.33</v>
+        <v>38.17</v>
       </c>
       <c r="C7" s="2">
         <v>5</v>
       </c>
       <c r="D7" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2">
         <v>5</v>
       </c>
       <c r="H7" s="2">
-        <v>55.56</v>
+        <v>33.590000000000003</v>
       </c>
       <c r="I7" s="2">
         <v>5</v>
       </c>
       <c r="J7" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -607,32 +607,32 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>88.89</v>
+        <v>45.8</v>
       </c>
       <c r="C8" s="2">
         <v>6</v>
       </c>
       <c r="D8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2">
         <v>6</v>
       </c>
       <c r="H8" s="2">
-        <v>66.67</v>
+        <v>35.880000000000003</v>
       </c>
       <c r="I8" s="2">
         <v>6</v>
       </c>
       <c r="J8" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K8" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -640,32 +640,32 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>94.44</v>
+        <v>52.67</v>
       </c>
       <c r="C9" s="2">
         <v>7</v>
       </c>
       <c r="D9" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2">
         <v>7</v>
       </c>
       <c r="H9" s="2">
-        <v>77.78</v>
+        <v>38.17</v>
       </c>
       <c r="I9" s="2">
         <v>7</v>
       </c>
       <c r="J9" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K9" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -673,32 +673,32 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>94.44</v>
+        <v>58.02</v>
       </c>
       <c r="C10" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2">
         <v>8</v>
       </c>
       <c r="H10" s="2">
-        <v>88.89</v>
+        <v>39.69</v>
       </c>
       <c r="I10" s="2">
         <v>8</v>
       </c>
       <c r="J10" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K10" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -706,13 +706,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>94.44</v>
+        <v>62.6</v>
       </c>
       <c r="C11" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D11" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="2">
         <v>7</v>
@@ -722,16 +722,16 @@
         <v>9</v>
       </c>
       <c r="H11" s="2">
-        <v>94.44</v>
+        <v>47.33</v>
       </c>
       <c r="I11" s="2">
         <v>9</v>
       </c>
       <c r="J11" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K11" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -739,117 +739,950 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>94.44</v>
+        <v>65.650000000000006</v>
       </c>
       <c r="C12" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D12" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2">
         <v>10</v>
       </c>
       <c r="H12" s="2">
-        <v>94.44</v>
+        <v>53.44</v>
       </c>
       <c r="I12" s="2">
+        <v>10</v>
+      </c>
+      <c r="J12" s="2">
+        <v>8</v>
+      </c>
+      <c r="K12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2">
+        <v>68.7</v>
+      </c>
+      <c r="C13" s="2">
+        <v>11</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2">
+        <v>10</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2">
+        <v>11</v>
+      </c>
+      <c r="H13" s="2">
+        <v>58.02</v>
+      </c>
+      <c r="I13" s="2">
+        <v>11</v>
+      </c>
+      <c r="J13" s="2">
+        <v>8</v>
+      </c>
+      <c r="K13" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2">
+        <v>71.760000000000005</v>
+      </c>
+      <c r="C14" s="2">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2">
+        <v>12</v>
+      </c>
+      <c r="H14" s="2">
+        <v>62.6</v>
+      </c>
+      <c r="I14" s="2">
+        <v>12</v>
+      </c>
+      <c r="J14" s="2">
+        <v>8</v>
+      </c>
+      <c r="K14" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>13</v>
+      </c>
+      <c r="B15" s="2">
+        <v>74.05</v>
+      </c>
+      <c r="C15" s="2">
+        <v>13</v>
+      </c>
+      <c r="D15" s="2">
+        <v>2</v>
+      </c>
+      <c r="E15" s="2">
+        <v>11</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2">
+        <v>13</v>
+      </c>
+      <c r="H15" s="2">
+        <v>66.41</v>
+      </c>
+      <c r="I15" s="2">
+        <v>13</v>
+      </c>
+      <c r="J15" s="2">
+        <v>8</v>
+      </c>
+      <c r="K15" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2">
+        <v>76.34</v>
+      </c>
+      <c r="C16" s="2">
+        <v>14</v>
+      </c>
+      <c r="D16" s="2">
+        <v>2</v>
+      </c>
+      <c r="E16" s="2">
+        <v>12</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2">
+        <v>14</v>
+      </c>
+      <c r="H16" s="2">
+        <v>69.47</v>
+      </c>
+      <c r="I16" s="2">
+        <v>14</v>
+      </c>
+      <c r="J16" s="2">
+        <v>8</v>
+      </c>
+      <c r="K16" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>15</v>
+      </c>
+      <c r="B17" s="2">
+        <v>78.63</v>
+      </c>
+      <c r="C17" s="2">
+        <v>15</v>
+      </c>
+      <c r="D17" s="2">
+        <v>2</v>
+      </c>
+      <c r="E17" s="2">
+        <v>13</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2">
+        <v>15</v>
+      </c>
+      <c r="H17" s="2">
+        <v>71.760000000000005</v>
+      </c>
+      <c r="I17" s="2">
+        <v>15</v>
+      </c>
+      <c r="J17" s="2">
+        <v>8</v>
+      </c>
+      <c r="K17" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>16</v>
+      </c>
+      <c r="B18" s="2">
+        <v>80.92</v>
+      </c>
+      <c r="C18" s="2">
+        <v>16</v>
+      </c>
+      <c r="D18" s="2">
+        <v>2</v>
+      </c>
+      <c r="E18" s="2">
+        <v>14</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2">
+        <v>16</v>
+      </c>
+      <c r="H18" s="2">
+        <v>74.05</v>
+      </c>
+      <c r="I18" s="2">
+        <v>16</v>
+      </c>
+      <c r="J18" s="2">
+        <v>8</v>
+      </c>
+      <c r="K18" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2">
+        <v>83.21</v>
+      </c>
+      <c r="C19" s="2">
+        <v>17</v>
+      </c>
+      <c r="D19" s="2">
+        <v>2</v>
+      </c>
+      <c r="E19" s="2">
+        <v>15</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2">
+        <v>17</v>
+      </c>
+      <c r="H19" s="2">
+        <v>76.34</v>
+      </c>
+      <c r="I19" s="2">
+        <v>17</v>
+      </c>
+      <c r="J19" s="2">
+        <v>8</v>
+      </c>
+      <c r="K19" s="2">
         <v>9</v>
       </c>
-      <c r="J12" s="2">
-        <v>4</v>
-      </c>
-      <c r="K12" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>18</v>
+      </c>
+      <c r="B20" s="2">
+        <v>83.97</v>
+      </c>
+      <c r="C20" s="2">
+        <v>18</v>
+      </c>
+      <c r="D20" s="2">
+        <v>2</v>
+      </c>
+      <c r="E20" s="2">
+        <v>16</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2">
+        <v>18</v>
+      </c>
+      <c r="H20" s="2">
+        <v>78.63</v>
+      </c>
+      <c r="I20" s="2">
+        <v>18</v>
+      </c>
+      <c r="J20" s="2">
+        <v>8</v>
+      </c>
+      <c r="K20" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2">
+        <v>84.73</v>
+      </c>
+      <c r="C21" s="2">
+        <v>19</v>
+      </c>
+      <c r="D21" s="2">
+        <v>2</v>
+      </c>
+      <c r="E21" s="2">
+        <v>17</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2">
+        <v>19</v>
+      </c>
+      <c r="H21" s="2">
+        <v>80.92</v>
+      </c>
+      <c r="I21" s="2">
+        <v>19</v>
+      </c>
+      <c r="J21" s="2">
+        <v>8</v>
+      </c>
+      <c r="K21" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2">
+        <v>85.5</v>
+      </c>
+      <c r="C22" s="2">
+        <v>20</v>
+      </c>
+      <c r="D22" s="2">
+        <v>2</v>
+      </c>
+      <c r="E22" s="2">
+        <v>18</v>
+      </c>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2">
+        <v>20</v>
+      </c>
+      <c r="H22" s="2">
+        <v>82.44</v>
+      </c>
+      <c r="I22" s="2">
+        <v>20</v>
+      </c>
+      <c r="J22" s="2">
+        <v>8</v>
+      </c>
+      <c r="K22" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2">
+        <v>86.26</v>
+      </c>
+      <c r="C23" s="2">
+        <v>21</v>
+      </c>
+      <c r="D23" s="2">
+        <v>2</v>
+      </c>
+      <c r="E23" s="2">
+        <v>19</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2">
+        <v>21</v>
+      </c>
+      <c r="H23" s="2">
+        <v>83.21</v>
+      </c>
+      <c r="I23" s="2">
+        <v>21</v>
+      </c>
+      <c r="J23" s="2">
+        <v>8</v>
+      </c>
+      <c r="K23" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2">
+        <v>87.02</v>
+      </c>
+      <c r="C24" s="2">
+        <v>22</v>
+      </c>
+      <c r="D24" s="2">
+        <v>2</v>
+      </c>
+      <c r="E24" s="2">
+        <v>20</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2">
+        <v>22</v>
+      </c>
+      <c r="H24" s="2">
+        <v>83.97</v>
+      </c>
+      <c r="I24" s="2">
+        <v>22</v>
+      </c>
+      <c r="J24" s="2">
+        <v>8</v>
+      </c>
+      <c r="K24" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2">
+        <v>87.79</v>
+      </c>
+      <c r="C25" s="2">
+        <v>23</v>
+      </c>
+      <c r="D25" s="2">
+        <v>2</v>
+      </c>
+      <c r="E25" s="2">
+        <v>21</v>
+      </c>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2">
+        <v>23</v>
+      </c>
+      <c r="H25" s="2">
+        <v>84.73</v>
+      </c>
+      <c r="I25" s="2">
+        <v>23</v>
+      </c>
+      <c r="J25" s="2">
+        <v>8</v>
+      </c>
+      <c r="K25" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2">
+        <v>88.55</v>
+      </c>
+      <c r="C26" s="2">
+        <v>24</v>
+      </c>
+      <c r="D26" s="2">
+        <v>2</v>
+      </c>
+      <c r="E26" s="2">
+        <v>22</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2">
+        <v>24</v>
+      </c>
+      <c r="H26" s="2">
+        <v>85.5</v>
+      </c>
+      <c r="I26" s="2">
+        <v>24</v>
+      </c>
+      <c r="J26" s="2">
+        <v>8</v>
+      </c>
+      <c r="K26" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>25</v>
+      </c>
+      <c r="B27" s="2">
+        <v>89.31</v>
+      </c>
+      <c r="C27" s="2">
+        <v>25</v>
+      </c>
+      <c r="D27" s="2">
+        <v>2</v>
+      </c>
+      <c r="E27" s="2">
+        <v>23</v>
+      </c>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2">
+        <v>25</v>
+      </c>
+      <c r="H27" s="2">
+        <v>86.26</v>
+      </c>
+      <c r="I27" s="2">
+        <v>25</v>
+      </c>
+      <c r="J27" s="2">
+        <v>8</v>
+      </c>
+      <c r="K27" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2">
+        <v>90.08</v>
+      </c>
+      <c r="C28" s="2">
+        <v>26</v>
+      </c>
+      <c r="D28" s="2">
+        <v>2</v>
+      </c>
+      <c r="E28" s="2">
+        <v>24</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2">
+        <v>26</v>
+      </c>
+      <c r="H28" s="2">
+        <v>87.02</v>
+      </c>
+      <c r="I28" s="2">
+        <v>26</v>
+      </c>
+      <c r="J28" s="2">
+        <v>8</v>
+      </c>
+      <c r="K28" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2">
+        <v>90.84</v>
+      </c>
+      <c r="C29" s="2">
+        <v>27</v>
+      </c>
+      <c r="D29" s="2">
+        <v>2</v>
+      </c>
+      <c r="E29" s="2">
+        <v>25</v>
+      </c>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2">
+        <v>27</v>
+      </c>
+      <c r="H29" s="2">
+        <v>87.79</v>
+      </c>
+      <c r="I29" s="2">
+        <v>27</v>
+      </c>
+      <c r="J29" s="2">
+        <v>8</v>
+      </c>
+      <c r="K29" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2">
+        <v>91.6</v>
+      </c>
+      <c r="C30" s="2">
+        <v>28</v>
+      </c>
+      <c r="D30" s="2">
+        <v>2</v>
+      </c>
+      <c r="E30" s="2">
+        <v>26</v>
+      </c>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2">
+        <v>28</v>
+      </c>
+      <c r="H30" s="2">
+        <v>88.55</v>
+      </c>
+      <c r="I30" s="2">
+        <v>28</v>
+      </c>
+      <c r="J30" s="2">
+        <v>8</v>
+      </c>
+      <c r="K30" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2">
+        <v>92.37</v>
+      </c>
+      <c r="C31" s="2">
+        <v>29</v>
+      </c>
+      <c r="D31" s="2">
+        <v>2</v>
+      </c>
+      <c r="E31" s="2">
+        <v>27</v>
+      </c>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2">
+        <v>29</v>
+      </c>
+      <c r="H31" s="2">
+        <v>89.31</v>
+      </c>
+      <c r="I31" s="2">
+        <v>29</v>
+      </c>
+      <c r="J31" s="2">
+        <v>8</v>
+      </c>
+      <c r="K31" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2">
+        <v>93.13</v>
+      </c>
+      <c r="C32" s="2">
+        <v>30</v>
+      </c>
+      <c r="D32" s="2">
+        <v>2</v>
+      </c>
+      <c r="E32" s="2">
+        <v>28</v>
+      </c>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2">
+        <v>30</v>
+      </c>
+      <c r="H32" s="2">
+        <v>90.08</v>
+      </c>
+      <c r="I32" s="2">
+        <v>30</v>
+      </c>
+      <c r="J32" s="2">
+        <v>8</v>
+      </c>
+      <c r="K32" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2">
+        <v>93.89</v>
+      </c>
+      <c r="C33" s="2">
+        <v>31</v>
+      </c>
+      <c r="D33" s="2">
+        <v>2</v>
+      </c>
+      <c r="E33" s="2">
+        <v>29</v>
+      </c>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2">
+        <v>31</v>
+      </c>
+      <c r="H33" s="2">
+        <v>90.84</v>
+      </c>
+      <c r="I33" s="2">
+        <v>31</v>
+      </c>
+      <c r="J33" s="2">
+        <v>8</v>
+      </c>
+      <c r="K33" s="2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="2">
+        <v>32</v>
+      </c>
+      <c r="B34" s="2">
+        <v>94.66</v>
+      </c>
+      <c r="C34" s="2">
+        <v>32</v>
+      </c>
+      <c r="D34" s="2">
+        <v>2</v>
+      </c>
+      <c r="E34" s="2">
+        <v>30</v>
+      </c>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2">
+        <v>32</v>
+      </c>
+      <c r="H34" s="2">
+        <v>91.6</v>
+      </c>
+      <c r="I34" s="2">
+        <v>32</v>
+      </c>
+      <c r="J34" s="2">
+        <v>8</v>
+      </c>
+      <c r="K34" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="2">
+        <v>33</v>
+      </c>
+      <c r="B35" s="2">
+        <v>95.42</v>
+      </c>
+      <c r="C35" s="2">
+        <v>33</v>
+      </c>
+      <c r="D35" s="2">
+        <v>2</v>
+      </c>
+      <c r="E35" s="2">
+        <v>31</v>
+      </c>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2">
+        <v>33</v>
+      </c>
+      <c r="H35" s="2">
+        <v>92.37</v>
+      </c>
+      <c r="I35" s="2">
+        <v>33</v>
+      </c>
+      <c r="J35" s="2">
+        <v>8</v>
+      </c>
+      <c r="K35" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="2">
+        <v>34</v>
+      </c>
+      <c r="B36" s="2">
+        <v>96.18</v>
+      </c>
+      <c r="C36" s="2">
+        <v>34</v>
+      </c>
+      <c r="D36" s="2">
+        <v>2</v>
+      </c>
+      <c r="E36" s="2">
+        <v>32</v>
+      </c>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2">
+        <v>34</v>
+      </c>
+      <c r="H36" s="2">
+        <v>93.13</v>
+      </c>
+      <c r="I36" s="2">
+        <v>34</v>
+      </c>
+      <c r="J36" s="2">
+        <v>8</v>
+      </c>
+      <c r="K36" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="2">
+        <v>35</v>
+      </c>
+      <c r="B37" s="2">
+        <v>96.18</v>
+      </c>
+      <c r="C37" s="2">
+        <v>34</v>
+      </c>
+      <c r="D37" s="2">
+        <v>2</v>
+      </c>
+      <c r="E37" s="2">
+        <v>32</v>
+      </c>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2">
+        <v>35</v>
+      </c>
+      <c r="H37" s="2">
+        <v>93.89</v>
+      </c>
+      <c r="I37" s="2">
+        <v>35</v>
+      </c>
+      <c r="J37" s="2">
+        <v>8</v>
+      </c>
+      <c r="K37" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2">
+        <v>36</v>
+      </c>
+      <c r="H38" s="2">
+        <v>94.66</v>
+      </c>
+      <c r="I38" s="2">
+        <v>36</v>
+      </c>
+      <c r="J38" s="2">
+        <v>8</v>
+      </c>
+      <c r="K38" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2">
+        <v>37</v>
+      </c>
+      <c r="H39" s="2">
+        <v>95.42</v>
+      </c>
+      <c r="I39" s="2">
+        <v>37</v>
+      </c>
+      <c r="J39" s="2">
+        <v>8</v>
+      </c>
+      <c r="K39" s="2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2">
+        <v>38</v>
+      </c>
+      <c r="H40" s="2">
+        <v>96.18</v>
+      </c>
+      <c r="I40" s="2">
+        <v>38</v>
+      </c>
+      <c r="J40" s="2">
+        <v>8</v>
+      </c>
+      <c r="K40" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2">
+        <v>39</v>
+      </c>
+      <c r="H41" s="2">
+        <v>96.18</v>
+      </c>
+      <c r="I41" s="2">
+        <v>38</v>
+      </c>
+      <c r="J41" s="2">
+        <v>8</v>
+      </c>
+      <c r="K41" s="2">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>